<commit_message>
Corrigiendo errores y ajustando exportar maquinaria
</commit_message>
<xml_diff>
--- a/public/plantillas/11_PROG_UTILIZACION.xlsx
+++ b/public/plantillas/11_PROG_UTILIZACION.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ventura/Desktop/Programacion/recal-hse/public/plantillas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9A772BA-1754-D145-8D49-CF333BFC59CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CEE151A7-C6E4-954C-B36F-0C275D49B32E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="33600" windowHeight="21000" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -558,9 +558,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -618,15 +615,36 @@
     <xf numFmtId="0" fontId="15" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -636,26 +654,8 @@
     <xf numFmtId="0" fontId="8" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1389,93 +1389,93 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="60" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
-      <c r="E1" s="27"/>
-      <c r="F1" s="27"/>
-      <c r="G1" s="27"/>
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="26"/>
+      <c r="F1" s="26"/>
+      <c r="G1" s="26"/>
     </row>
     <row r="2" spans="1:20" ht="27" x14ac:dyDescent="0.15">
-      <c r="A2" s="28" t="s">
+      <c r="A2" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="29"/>
-      <c r="C2" s="29"/>
-      <c r="D2" s="32"/>
-      <c r="E2" s="28" t="s">
+      <c r="B2" s="28"/>
+      <c r="C2" s="28"/>
+      <c r="D2" s="31"/>
+      <c r="E2" s="27" t="s">
         <v>51</v>
       </c>
-      <c r="F2" s="29"/>
-      <c r="G2" s="29"/>
+      <c r="F2" s="28"/>
+      <c r="G2" s="28"/>
     </row>
     <row r="3" spans="1:20" ht="49" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A3" s="28" t="s">
+      <c r="A3" s="27" t="s">
         <v>45</v>
       </c>
-      <c r="B3" s="29"/>
-      <c r="C3" s="29"/>
-      <c r="D3" s="32"/>
-      <c r="E3" s="30"/>
-      <c r="F3" s="31"/>
-      <c r="G3" s="31"/>
+      <c r="B3" s="28"/>
+      <c r="C3" s="28"/>
+      <c r="D3" s="31"/>
+      <c r="E3" s="29"/>
+      <c r="F3" s="30"/>
+      <c r="G3" s="30"/>
     </row>
     <row r="4" spans="1:20" ht="50" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A4" s="18" t="s">
+      <c r="A4" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="18" t="s">
+      <c r="B4" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="19" t="s">
+      <c r="C4" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="D4" s="18" t="s">
+      <c r="D4" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="E4" s="18" t="s">
+      <c r="E4" s="17" t="s">
         <v>47</v>
       </c>
-      <c r="F4" s="20" t="s">
+      <c r="F4" s="19" t="s">
         <v>46</v>
       </c>
-      <c r="G4" s="21" t="s">
+      <c r="G4" s="20" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="5" spans="1:20" ht="180" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A5" s="14"/>
-      <c r="B5" s="15"/>
-      <c r="C5" s="14"/>
-      <c r="D5" s="16"/>
-      <c r="E5" s="14"/>
-      <c r="F5" s="17"/>
-      <c r="G5" s="13"/>
+      <c r="A5" s="13"/>
+      <c r="B5" s="14"/>
+      <c r="C5" s="13"/>
+      <c r="D5" s="15"/>
+      <c r="E5" s="13"/>
+      <c r="F5" s="16"/>
+      <c r="G5" s="45"/>
     </row>
     <row r="6" spans="1:20" ht="69" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A6" s="22" t="s">
+      <c r="A6" s="21" t="s">
         <v>49</v>
       </c>
-      <c r="B6" s="22"/>
-      <c r="C6" s="22"/>
-      <c r="D6" s="22"/>
-      <c r="E6" s="22"/>
-      <c r="F6" s="22"/>
-      <c r="G6" s="22"/>
+      <c r="B6" s="21"/>
+      <c r="C6" s="21"/>
+      <c r="D6" s="21"/>
+      <c r="E6" s="21"/>
+      <c r="F6" s="21"/>
+      <c r="G6" s="21"/>
     </row>
     <row r="7" spans="1:20" ht="13.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A7" s="23" t="s">
+      <c r="A7" s="22" t="s">
         <v>48</v>
       </c>
-      <c r="B7" s="24"/>
-      <c r="C7" s="24"/>
-      <c r="D7" s="24"/>
-      <c r="E7" s="24"/>
-      <c r="F7" s="24"/>
-      <c r="G7" s="24"/>
+      <c r="B7" s="23"/>
+      <c r="C7" s="23"/>
+      <c r="D7" s="23"/>
+      <c r="E7" s="23"/>
+      <c r="F7" s="23"/>
+      <c r="G7" s="23"/>
       <c r="I7" s="12"/>
       <c r="J7" s="12"/>
       <c r="K7" s="12"/>
@@ -1490,15 +1490,15 @@
       <c r="T7" s="12"/>
     </row>
     <row r="8" spans="1:20" ht="81" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="25" t="s">
+      <c r="A8" s="24" t="s">
         <v>50</v>
       </c>
-      <c r="B8" s="26"/>
-      <c r="C8" s="26"/>
-      <c r="D8" s="26"/>
-      <c r="E8" s="26"/>
-      <c r="F8" s="26"/>
-      <c r="G8" s="26"/>
+      <c r="B8" s="25"/>
+      <c r="C8" s="25"/>
+      <c r="D8" s="25"/>
+      <c r="E8" s="25"/>
+      <c r="F8" s="25"/>
+      <c r="G8" s="25"/>
     </row>
     <row r="9" spans="1:20" ht="30.75" customHeight="1" x14ac:dyDescent="0.15"/>
     <row r="10" spans="1:20" ht="52.5" customHeight="1" x14ac:dyDescent="0.15"/>
@@ -2518,59 +2518,59 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="60" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
-      <c r="E1" s="27"/>
-      <c r="F1" s="27"/>
-      <c r="G1" s="27"/>
-      <c r="H1" s="27"/>
-      <c r="I1" s="27"/>
-      <c r="J1" s="27"/>
-      <c r="K1" s="27"/>
-      <c r="L1" s="27"/>
-      <c r="M1" s="27"/>
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="26"/>
+      <c r="F1" s="26"/>
+      <c r="G1" s="26"/>
+      <c r="H1" s="26"/>
+      <c r="I1" s="26"/>
+      <c r="J1" s="26"/>
+      <c r="K1" s="26"/>
+      <c r="L1" s="26"/>
+      <c r="M1" s="26"/>
     </row>
     <row r="2" spans="1:26" ht="20" x14ac:dyDescent="0.15">
-      <c r="A2" s="43" t="s">
+      <c r="A2" s="32" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="43"/>
-      <c r="C2" s="43"/>
-      <c r="D2" s="43"/>
-      <c r="E2" s="43"/>
-      <c r="F2" s="44" t="s">
+      <c r="B2" s="32"/>
+      <c r="C2" s="32"/>
+      <c r="D2" s="32"/>
+      <c r="E2" s="32"/>
+      <c r="F2" s="33" t="s">
         <v>44</v>
       </c>
-      <c r="G2" s="44"/>
-      <c r="H2" s="44"/>
-      <c r="I2" s="44"/>
-      <c r="J2" s="44"/>
-      <c r="K2" s="44"/>
-      <c r="L2" s="44"/>
-      <c r="M2" s="44"/>
+      <c r="G2" s="33"/>
+      <c r="H2" s="33"/>
+      <c r="I2" s="33"/>
+      <c r="J2" s="33"/>
+      <c r="K2" s="33"/>
+      <c r="L2" s="33"/>
+      <c r="M2" s="33"/>
     </row>
     <row r="3" spans="1:26" ht="26.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A3" s="43" t="s">
+      <c r="A3" s="32" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="43"/>
-      <c r="C3" s="43"/>
-      <c r="D3" s="43"/>
-      <c r="E3" s="43"/>
-      <c r="F3" s="45" t="s">
+      <c r="B3" s="32"/>
+      <c r="C3" s="32"/>
+      <c r="D3" s="32"/>
+      <c r="E3" s="32"/>
+      <c r="F3" s="34" t="s">
         <v>3</v>
       </c>
-      <c r="G3" s="45"/>
-      <c r="H3" s="45"/>
-      <c r="I3" s="45"/>
-      <c r="J3" s="45"/>
-      <c r="K3" s="45"/>
-      <c r="L3" s="45"/>
-      <c r="M3" s="45"/>
+      <c r="G3" s="34"/>
+      <c r="H3" s="34"/>
+      <c r="I3" s="34"/>
+      <c r="J3" s="34"/>
+      <c r="K3" s="34"/>
+      <c r="L3" s="34"/>
+      <c r="M3" s="34"/>
     </row>
     <row r="4" spans="1:26" ht="36.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="2" t="s">
@@ -2588,20 +2588,20 @@
       <c r="E4" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="F4" s="41" t="s">
+      <c r="F4" s="35" t="s">
         <v>9</v>
       </c>
-      <c r="G4" s="41"/>
-      <c r="H4" s="41" t="s">
+      <c r="G4" s="35"/>
+      <c r="H4" s="35" t="s">
         <v>10</v>
       </c>
-      <c r="I4" s="41"/>
-      <c r="J4" s="42" t="s">
+      <c r="I4" s="35"/>
+      <c r="J4" s="36" t="s">
         <v>11</v>
       </c>
-      <c r="K4" s="42"/>
-      <c r="L4" s="42"/>
-      <c r="M4" s="42"/>
+      <c r="K4" s="36"/>
+      <c r="L4" s="36"/>
+      <c r="M4" s="36"/>
     </row>
     <row r="5" spans="1:26" ht="207.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="4">
@@ -2619,18 +2619,18 @@
       <c r="E5" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F5" s="39" t="s">
+      <c r="F5" s="37" t="s">
         <v>16</v>
       </c>
-      <c r="G5" s="39"/>
-      <c r="H5" s="34" t="s">
+      <c r="G5" s="37"/>
+      <c r="H5" s="38" t="s">
         <v>17</v>
       </c>
-      <c r="I5" s="34"/>
-      <c r="J5" s="40"/>
-      <c r="K5" s="40"/>
-      <c r="L5" s="40"/>
-      <c r="M5" s="40"/>
+      <c r="I5" s="38"/>
+      <c r="J5" s="39"/>
+      <c r="K5" s="39"/>
+      <c r="L5" s="39"/>
+      <c r="M5" s="39"/>
     </row>
     <row r="6" spans="1:26" ht="207.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="4">
@@ -2648,18 +2648,18 @@
       <c r="E6" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F6" s="39" t="s">
+      <c r="F6" s="37" t="s">
         <v>16</v>
       </c>
-      <c r="G6" s="39"/>
-      <c r="H6" s="34" t="s">
+      <c r="G6" s="37"/>
+      <c r="H6" s="38" t="s">
         <v>17</v>
       </c>
-      <c r="I6" s="34"/>
-      <c r="J6" s="40"/>
-      <c r="K6" s="40"/>
-      <c r="L6" s="40"/>
-      <c r="M6" s="40"/>
+      <c r="I6" s="38"/>
+      <c r="J6" s="39"/>
+      <c r="K6" s="39"/>
+      <c r="L6" s="39"/>
+      <c r="M6" s="39"/>
     </row>
     <row r="7" spans="1:26" ht="207.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="4">
@@ -2677,18 +2677,18 @@
       <c r="E7" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F7" s="39" t="s">
+      <c r="F7" s="37" t="s">
         <v>22</v>
       </c>
-      <c r="G7" s="39"/>
-      <c r="H7" s="34" t="s">
+      <c r="G7" s="37"/>
+      <c r="H7" s="38" t="s">
         <v>17</v>
       </c>
-      <c r="I7" s="34"/>
-      <c r="J7" s="40"/>
-      <c r="K7" s="40"/>
-      <c r="L7" s="40"/>
-      <c r="M7" s="40"/>
+      <c r="I7" s="38"/>
+      <c r="J7" s="39"/>
+      <c r="K7" s="39"/>
+      <c r="L7" s="39"/>
+      <c r="M7" s="39"/>
     </row>
     <row r="8" spans="1:26" ht="208.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="4">
@@ -2706,18 +2706,18 @@
       <c r="E8" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F8" s="34" t="s">
+      <c r="F8" s="38" t="s">
         <v>26</v>
       </c>
-      <c r="G8" s="34"/>
-      <c r="H8" s="34" t="s">
+      <c r="G8" s="38"/>
+      <c r="H8" s="38" t="s">
         <v>17</v>
       </c>
-      <c r="I8" s="34"/>
-      <c r="J8" s="40"/>
-      <c r="K8" s="40"/>
-      <c r="L8" s="40"/>
-      <c r="M8" s="40"/>
+      <c r="I8" s="38"/>
+      <c r="J8" s="39"/>
+      <c r="K8" s="39"/>
+      <c r="L8" s="39"/>
+      <c r="M8" s="39"/>
     </row>
     <row r="9" spans="1:26" ht="208.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="4">
@@ -2735,18 +2735,18 @@
       <c r="E9" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F9" s="39" t="s">
+      <c r="F9" s="37" t="s">
         <v>30</v>
       </c>
-      <c r="G9" s="39"/>
-      <c r="H9" s="34" t="s">
+      <c r="G9" s="37"/>
+      <c r="H9" s="38" t="s">
         <v>17</v>
       </c>
-      <c r="I9" s="34"/>
-      <c r="J9" s="35"/>
-      <c r="K9" s="35"/>
-      <c r="L9" s="35"/>
-      <c r="M9" s="35"/>
+      <c r="I9" s="38"/>
+      <c r="J9" s="40"/>
+      <c r="K9" s="40"/>
+      <c r="L9" s="40"/>
+      <c r="M9" s="40"/>
     </row>
     <row r="10" spans="1:26" ht="208.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="4">
@@ -2764,18 +2764,18 @@
       <c r="E10" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F10" s="39" t="s">
+      <c r="F10" s="37" t="s">
         <v>30</v>
       </c>
-      <c r="G10" s="39"/>
-      <c r="H10" s="34" t="s">
+      <c r="G10" s="37"/>
+      <c r="H10" s="38" t="s">
         <v>17</v>
       </c>
-      <c r="I10" s="34"/>
-      <c r="J10" s="35"/>
-      <c r="K10" s="35"/>
-      <c r="L10" s="35"/>
-      <c r="M10" s="35"/>
+      <c r="I10" s="38"/>
+      <c r="J10" s="40"/>
+      <c r="K10" s="40"/>
+      <c r="L10" s="40"/>
+      <c r="M10" s="40"/>
     </row>
     <row r="11" spans="1:26" ht="208.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="4">
@@ -2793,18 +2793,18 @@
       <c r="E11" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F11" s="34" t="s">
+      <c r="F11" s="38" t="s">
         <v>36</v>
       </c>
-      <c r="G11" s="34"/>
-      <c r="H11" s="34" t="s">
+      <c r="G11" s="38"/>
+      <c r="H11" s="38" t="s">
         <v>17</v>
       </c>
-      <c r="I11" s="34"/>
-      <c r="J11" s="35"/>
-      <c r="K11" s="35"/>
-      <c r="L11" s="35"/>
-      <c r="M11" s="35"/>
+      <c r="I11" s="38"/>
+      <c r="J11" s="40"/>
+      <c r="K11" s="40"/>
+      <c r="L11" s="40"/>
+      <c r="M11" s="40"/>
     </row>
     <row r="12" spans="1:26" ht="208.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="4">
@@ -2822,54 +2822,54 @@
       <c r="E12" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F12" s="34" t="s">
+      <c r="F12" s="38" t="s">
         <v>36</v>
       </c>
-      <c r="G12" s="34"/>
-      <c r="H12" s="34" t="s">
+      <c r="G12" s="38"/>
+      <c r="H12" s="38" t="s">
         <v>17</v>
       </c>
-      <c r="I12" s="34"/>
-      <c r="J12" s="35"/>
-      <c r="K12" s="35"/>
-      <c r="L12" s="35"/>
-      <c r="M12" s="35"/>
+      <c r="I12" s="38"/>
+      <c r="J12" s="40"/>
+      <c r="K12" s="40"/>
+      <c r="L12" s="40"/>
+      <c r="M12" s="40"/>
     </row>
     <row r="13" spans="1:26" ht="69" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A13" s="36" t="s">
+      <c r="A13" s="42" t="s">
         <v>39</v>
       </c>
-      <c r="B13" s="36"/>
-      <c r="C13" s="36"/>
-      <c r="D13" s="36"/>
-      <c r="E13" s="36"/>
-      <c r="F13" s="36"/>
-      <c r="G13" s="36"/>
-      <c r="H13" s="36"/>
-      <c r="I13" s="36"/>
-      <c r="J13" s="36"/>
-      <c r="K13" s="36"/>
-      <c r="L13" s="36"/>
-      <c r="M13" s="36"/>
+      <c r="B13" s="42"/>
+      <c r="C13" s="42"/>
+      <c r="D13" s="42"/>
+      <c r="E13" s="42"/>
+      <c r="F13" s="42"/>
+      <c r="G13" s="42"/>
+      <c r="H13" s="42"/>
+      <c r="I13" s="42"/>
+      <c r="J13" s="42"/>
+      <c r="K13" s="42"/>
+      <c r="L13" s="42"/>
+      <c r="M13" s="42"/>
     </row>
     <row r="14" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A14" s="37" t="s">
+      <c r="A14" s="43" t="s">
         <v>40</v>
       </c>
-      <c r="B14" s="37"/>
-      <c r="C14" s="37"/>
-      <c r="D14" s="37"/>
-      <c r="E14" s="37"/>
-      <c r="F14" s="38" t="s">
+      <c r="B14" s="43"/>
+      <c r="C14" s="43"/>
+      <c r="D14" s="43"/>
+      <c r="E14" s="43"/>
+      <c r="F14" s="44" t="s">
         <v>41</v>
       </c>
-      <c r="G14" s="38"/>
-      <c r="H14" s="38"/>
-      <c r="I14" s="38"/>
-      <c r="J14" s="38"/>
-      <c r="K14" s="38"/>
-      <c r="L14" s="38"/>
-      <c r="M14" s="38"/>
+      <c r="G14" s="44"/>
+      <c r="H14" s="44"/>
+      <c r="I14" s="44"/>
+      <c r="J14" s="44"/>
+      <c r="K14" s="44"/>
+      <c r="L14" s="44"/>
+      <c r="M14" s="44"/>
       <c r="N14" s="12"/>
       <c r="O14" s="12"/>
       <c r="P14" s="12"/>
@@ -2885,23 +2885,23 @@
       <c r="Z14" s="12"/>
     </row>
     <row r="15" spans="1:26" ht="81" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A15" s="33" t="s">
+      <c r="A15" s="41" t="s">
         <v>42</v>
       </c>
-      <c r="B15" s="33"/>
-      <c r="C15" s="33"/>
-      <c r="D15" s="33"/>
-      <c r="E15" s="33"/>
-      <c r="F15" s="33" t="s">
+      <c r="B15" s="41"/>
+      <c r="C15" s="41"/>
+      <c r="D15" s="41"/>
+      <c r="E15" s="41"/>
+      <c r="F15" s="41" t="s">
         <v>43</v>
       </c>
-      <c r="G15" s="33"/>
-      <c r="H15" s="33"/>
-      <c r="I15" s="33"/>
-      <c r="J15" s="33"/>
-      <c r="K15" s="33"/>
-      <c r="L15" s="33"/>
-      <c r="M15" s="33"/>
+      <c r="G15" s="41"/>
+      <c r="H15" s="41"/>
+      <c r="I15" s="41"/>
+      <c r="J15" s="41"/>
+      <c r="K15" s="41"/>
+      <c r="L15" s="41"/>
+      <c r="M15" s="41"/>
     </row>
     <row r="16" spans="1:26" ht="30.75" customHeight="1" x14ac:dyDescent="0.15"/>
     <row r="17" ht="52.5" customHeight="1" x14ac:dyDescent="0.15"/>
@@ -3881,35 +3881,6 @@
     <row r="991" ht="13.5" customHeight="1" x14ac:dyDescent="0.15"/>
   </sheetData>
   <mergeCells count="37">
-    <mergeCell ref="A1:M1"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="F2:M2"/>
-    <mergeCell ref="A3:E3"/>
-    <mergeCell ref="F3:M3"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="H4:I4"/>
-    <mergeCell ref="J4:M4"/>
-    <mergeCell ref="F5:G5"/>
-    <mergeCell ref="H5:I5"/>
-    <mergeCell ref="J5:M5"/>
-    <mergeCell ref="F6:G6"/>
-    <mergeCell ref="H6:I6"/>
-    <mergeCell ref="J6:M6"/>
-    <mergeCell ref="F7:G7"/>
-    <mergeCell ref="H7:I7"/>
-    <mergeCell ref="J7:M7"/>
-    <mergeCell ref="F8:G8"/>
-    <mergeCell ref="H8:I8"/>
-    <mergeCell ref="J8:M8"/>
-    <mergeCell ref="F9:G9"/>
-    <mergeCell ref="H9:I9"/>
-    <mergeCell ref="J9:M9"/>
-    <mergeCell ref="F10:G10"/>
-    <mergeCell ref="H10:I10"/>
-    <mergeCell ref="J10:M10"/>
-    <mergeCell ref="F11:G11"/>
-    <mergeCell ref="H11:I11"/>
-    <mergeCell ref="J11:M11"/>
     <mergeCell ref="A15:E15"/>
     <mergeCell ref="F15:M15"/>
     <mergeCell ref="F12:G12"/>
@@ -3918,6 +3889,35 @@
     <mergeCell ref="A13:M13"/>
     <mergeCell ref="A14:E14"/>
     <mergeCell ref="F14:M14"/>
+    <mergeCell ref="F10:G10"/>
+    <mergeCell ref="H10:I10"/>
+    <mergeCell ref="J10:M10"/>
+    <mergeCell ref="F11:G11"/>
+    <mergeCell ref="H11:I11"/>
+    <mergeCell ref="J11:M11"/>
+    <mergeCell ref="F8:G8"/>
+    <mergeCell ref="H8:I8"/>
+    <mergeCell ref="J8:M8"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="H9:I9"/>
+    <mergeCell ref="J9:M9"/>
+    <mergeCell ref="F6:G6"/>
+    <mergeCell ref="H6:I6"/>
+    <mergeCell ref="J6:M6"/>
+    <mergeCell ref="F7:G7"/>
+    <mergeCell ref="H7:I7"/>
+    <mergeCell ref="J7:M7"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="H4:I4"/>
+    <mergeCell ref="J4:M4"/>
+    <mergeCell ref="F5:G5"/>
+    <mergeCell ref="H5:I5"/>
+    <mergeCell ref="J5:M5"/>
+    <mergeCell ref="A1:M1"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="F2:M2"/>
+    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="F3:M3"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.23611111111111099" right="0.23611111111111099" top="0.74791666666666701" bottom="0.74791666666666701" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Agregando columna de baja de maquinaria
</commit_message>
<xml_diff>
--- a/public/plantillas/11_PROG_UTILIZACION.xlsx
+++ b/public/plantillas/11_PROG_UTILIZACION.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ventura/Desktop/Programacion/recal-hse/public/plantillas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{504A741B-9C59-1545-8671-64CC2E40361A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A43E844-1FB9-3C42-BD7D-EB305A9EF62F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="33600" windowHeight="21000" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="MANTENIMIENTO MARZO 2024" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'MANTENIMIENTO FEBRERO 2024'!$A$1:$G$8</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'MANTENIMIENTO FEBRERO 2024'!$A$1:$H$8</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'MANTENIMIENTO MARZO 2024'!$A$1:$M$16</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'MANTENIMIENTO FEBRERO 2024'!$1:$4</definedName>
   </definedNames>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="56">
   <si>
     <t>PROGRAMA DE UTILIZACIÓN DE MAQUINARIA Y EQUIPO</t>
   </si>
@@ -183,9 +183,6 @@
     <t>CONTRATISTA: RECAL ESTRUCTURAS</t>
   </si>
   <si>
-    <t>FECHA DE INGRESO A OBRA</t>
-  </si>
-  <si>
     <t>NUMERO ECONOMICO</t>
   </si>
   <si>
@@ -209,6 +206,12 @@
   </si>
   <si>
     <t>PROYECTO: REHABILITACION, SUSTITUCION Y/O MODERNIZACION DE 526 PUENTES DE LA LINEA K</t>
+  </si>
+  <si>
+    <t>INGRESO A OBRA</t>
+  </si>
+  <si>
+    <t>BAJA DE OBRA</t>
   </si>
 </sst>
 </file>
@@ -372,7 +375,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -465,34 +468,6 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
         <color auto="1"/>
       </left>
       <right/>
@@ -568,18 +543,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="13" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="14" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
     <xf numFmtId="0" fontId="16" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -589,44 +552,95 @@
     <xf numFmtId="0" fontId="16" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="3" fontId="14" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="13" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="16" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -635,45 +649,6 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1393,7 +1368,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:T984"/>
+  <dimension ref="A1:U984"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.5" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="9.83203125" customWidth="1"/>
@@ -1401,15 +1376,15 @@
     <col min="3" max="3" width="59.5" customWidth="1"/>
     <col min="4" max="4" width="38.83203125" customWidth="1"/>
     <col min="5" max="5" width="43.5" customWidth="1"/>
-    <col min="6" max="6" width="40.83203125" customWidth="1"/>
-    <col min="7" max="7" width="30.83203125" customWidth="1"/>
-    <col min="8" max="8" width="119.5" customWidth="1"/>
-    <col min="9" max="20" width="10.5" customWidth="1"/>
+    <col min="6" max="7" width="40.83203125" customWidth="1"/>
+    <col min="8" max="8" width="30.83203125" customWidth="1"/>
+    <col min="9" max="9" width="119.5" customWidth="1"/>
+    <col min="10" max="21" width="10.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" ht="60" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:21" ht="60" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A1" s="27" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B1" s="27"/>
       <c r="C1" s="27"/>
@@ -1417,21 +1392,23 @@
       <c r="E1" s="27"/>
       <c r="F1" s="27"/>
       <c r="G1" s="27"/>
+      <c r="H1" s="27"/>
     </row>
-    <row r="2" spans="1:20" ht="27" x14ac:dyDescent="0.15">
-      <c r="A2" s="46" t="s">
-        <v>54</v>
-      </c>
-      <c r="B2" s="47"/>
-      <c r="C2" s="47"/>
-      <c r="D2" s="48"/>
+    <row r="2" spans="1:21" ht="27" x14ac:dyDescent="0.15">
+      <c r="A2" s="33" t="s">
+        <v>53</v>
+      </c>
+      <c r="B2" s="34"/>
+      <c r="C2" s="34"/>
+      <c r="D2" s="35"/>
       <c r="E2" s="28" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F2" s="29"/>
       <c r="G2" s="29"/>
+      <c r="H2" s="29"/>
     </row>
-    <row r="3" spans="1:20" ht="49" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="3" spans="1:21" ht="49" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="28" t="s">
         <v>45</v>
       </c>
@@ -1441,42 +1418,47 @@
       <c r="E3" s="30"/>
       <c r="F3" s="31"/>
       <c r="G3" s="31"/>
+      <c r="H3" s="31"/>
     </row>
-    <row r="4" spans="1:20" ht="50" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A4" s="17" t="s">
+    <row r="4" spans="1:21" ht="50" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A4" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="17" t="s">
+      <c r="B4" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="18" t="s">
+      <c r="C4" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="D4" s="17" t="s">
+      <c r="D4" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="E4" s="17" t="s">
-        <v>47</v>
-      </c>
-      <c r="F4" s="19" t="s">
+      <c r="E4" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="G4" s="20" t="s">
-        <v>52</v>
+      <c r="F4" s="15" t="s">
+        <v>54</v>
+      </c>
+      <c r="G4" s="15" t="s">
+        <v>55</v>
+      </c>
+      <c r="H4" s="18" t="s">
+        <v>51</v>
       </c>
     </row>
-    <row r="5" spans="1:20" ht="157" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A5" s="13"/>
-      <c r="B5" s="14"/>
-      <c r="C5" s="13"/>
-      <c r="D5" s="15"/>
-      <c r="E5" s="13"/>
-      <c r="F5" s="16"/>
-      <c r="G5" s="21"/>
+    <row r="5" spans="1:21" ht="157" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A5" s="19"/>
+      <c r="B5" s="20"/>
+      <c r="C5" s="19"/>
+      <c r="D5" s="21"/>
+      <c r="E5" s="19"/>
+      <c r="F5" s="17"/>
+      <c r="G5" s="17"/>
+      <c r="H5" s="16"/>
     </row>
-    <row r="6" spans="1:20" ht="69" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="6" spans="1:21" ht="69" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="22" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B6" s="22"/>
       <c r="C6" s="22"/>
@@ -1484,10 +1466,11 @@
       <c r="E6" s="22"/>
       <c r="F6" s="22"/>
       <c r="G6" s="22"/>
+      <c r="H6" s="22"/>
     </row>
-    <row r="7" spans="1:20" ht="13.5" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="7" spans="1:21" ht="13.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="23" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B7" s="24"/>
       <c r="C7" s="24"/>
@@ -1495,7 +1478,7 @@
       <c r="E7" s="24"/>
       <c r="F7" s="24"/>
       <c r="G7" s="24"/>
-      <c r="I7" s="12"/>
+      <c r="H7" s="24"/>
       <c r="J7" s="12"/>
       <c r="K7" s="12"/>
       <c r="L7" s="12"/>
@@ -1507,10 +1490,11 @@
       <c r="R7" s="12"/>
       <c r="S7" s="12"/>
       <c r="T7" s="12"/>
+      <c r="U7" s="12"/>
     </row>
-    <row r="8" spans="1:20" ht="81" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:21" ht="81" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="25" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B8" s="26"/>
       <c r="C8" s="26"/>
@@ -1518,15 +1502,16 @@
       <c r="E8" s="26"/>
       <c r="F8" s="26"/>
       <c r="G8" s="26"/>
+      <c r="H8" s="26"/>
     </row>
-    <row r="9" spans="1:20" ht="30.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="10" spans="1:20" ht="52.5" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="11" spans="1:20" ht="8.25" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="12" spans="1:20" ht="13.5" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="13" spans="1:20" ht="13.5" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="14" spans="1:20" ht="13.5" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="15" spans="1:20" ht="13.5" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="16" spans="1:20" ht="13.5" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="9" spans="1:21" ht="30.75" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="10" spans="1:21" ht="52.5" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="11" spans="1:21" ht="8.25" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="12" spans="1:21" ht="13.5" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="13" spans="1:21" ht="13.5" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="14" spans="1:21" ht="13.5" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="15" spans="1:21" ht="13.5" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="16" spans="1:21" ht="13.5" customHeight="1" x14ac:dyDescent="0.15"/>
     <row r="17" ht="13.5" customHeight="1" x14ac:dyDescent="0.15"/>
     <row r="18" ht="13.5" customHeight="1" x14ac:dyDescent="0.15"/>
     <row r="19" ht="13.5" customHeight="1" x14ac:dyDescent="0.15"/>
@@ -2497,12 +2482,12 @@
     <row r="984" ht="13.5" customHeight="1" x14ac:dyDescent="0.15"/>
   </sheetData>
   <mergeCells count="8">
-    <mergeCell ref="A6:G6"/>
-    <mergeCell ref="A7:G7"/>
-    <mergeCell ref="A8:G8"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="E2:G2"/>
-    <mergeCell ref="E3:G3"/>
+    <mergeCell ref="A6:H6"/>
+    <mergeCell ref="A7:H7"/>
+    <mergeCell ref="A8:H8"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="E2:H2"/>
+    <mergeCell ref="E3:H3"/>
     <mergeCell ref="A3:D3"/>
     <mergeCell ref="A2:D2"/>
   </mergeCells>
@@ -2554,42 +2539,42 @@
       <c r="M1" s="27"/>
     </row>
     <row r="2" spans="1:26" ht="20" x14ac:dyDescent="0.15">
-      <c r="A2" s="33" t="s">
+      <c r="A2" s="46" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="33"/>
-      <c r="C2" s="33"/>
-      <c r="D2" s="33"/>
-      <c r="E2" s="33"/>
-      <c r="F2" s="34" t="s">
+      <c r="B2" s="46"/>
+      <c r="C2" s="46"/>
+      <c r="D2" s="46"/>
+      <c r="E2" s="46"/>
+      <c r="F2" s="47" t="s">
         <v>44</v>
       </c>
-      <c r="G2" s="34"/>
-      <c r="H2" s="34"/>
-      <c r="I2" s="34"/>
-      <c r="J2" s="34"/>
-      <c r="K2" s="34"/>
-      <c r="L2" s="34"/>
-      <c r="M2" s="34"/>
+      <c r="G2" s="47"/>
+      <c r="H2" s="47"/>
+      <c r="I2" s="47"/>
+      <c r="J2" s="47"/>
+      <c r="K2" s="47"/>
+      <c r="L2" s="47"/>
+      <c r="M2" s="47"/>
     </row>
     <row r="3" spans="1:26" ht="26.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A3" s="33" t="s">
+      <c r="A3" s="46" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="33"/>
-      <c r="C3" s="33"/>
-      <c r="D3" s="33"/>
-      <c r="E3" s="33"/>
-      <c r="F3" s="35" t="s">
+      <c r="B3" s="46"/>
+      <c r="C3" s="46"/>
+      <c r="D3" s="46"/>
+      <c r="E3" s="46"/>
+      <c r="F3" s="48" t="s">
         <v>3</v>
       </c>
-      <c r="G3" s="35"/>
-      <c r="H3" s="35"/>
-      <c r="I3" s="35"/>
-      <c r="J3" s="35"/>
-      <c r="K3" s="35"/>
-      <c r="L3" s="35"/>
-      <c r="M3" s="35"/>
+      <c r="G3" s="48"/>
+      <c r="H3" s="48"/>
+      <c r="I3" s="48"/>
+      <c r="J3" s="48"/>
+      <c r="K3" s="48"/>
+      <c r="L3" s="48"/>
+      <c r="M3" s="48"/>
     </row>
     <row r="4" spans="1:26" ht="36.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="2" t="s">
@@ -2607,20 +2592,20 @@
       <c r="E4" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="F4" s="36" t="s">
+      <c r="F4" s="44" t="s">
         <v>9</v>
       </c>
-      <c r="G4" s="36"/>
-      <c r="H4" s="36" t="s">
+      <c r="G4" s="44"/>
+      <c r="H4" s="44" t="s">
         <v>10</v>
       </c>
-      <c r="I4" s="36"/>
-      <c r="J4" s="37" t="s">
+      <c r="I4" s="44"/>
+      <c r="J4" s="45" t="s">
         <v>11</v>
       </c>
-      <c r="K4" s="37"/>
-      <c r="L4" s="37"/>
-      <c r="M4" s="37"/>
+      <c r="K4" s="45"/>
+      <c r="L4" s="45"/>
+      <c r="M4" s="45"/>
     </row>
     <row r="5" spans="1:26" ht="207.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="4">
@@ -2638,18 +2623,18 @@
       <c r="E5" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F5" s="38" t="s">
+      <c r="F5" s="42" t="s">
         <v>16</v>
       </c>
-      <c r="G5" s="38"/>
-      <c r="H5" s="39" t="s">
+      <c r="G5" s="42"/>
+      <c r="H5" s="37" t="s">
         <v>17</v>
       </c>
-      <c r="I5" s="39"/>
-      <c r="J5" s="40"/>
-      <c r="K5" s="40"/>
-      <c r="L5" s="40"/>
-      <c r="M5" s="40"/>
+      <c r="I5" s="37"/>
+      <c r="J5" s="43"/>
+      <c r="K5" s="43"/>
+      <c r="L5" s="43"/>
+      <c r="M5" s="43"/>
     </row>
     <row r="6" spans="1:26" ht="207.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="4">
@@ -2667,18 +2652,18 @@
       <c r="E6" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F6" s="38" t="s">
+      <c r="F6" s="42" t="s">
         <v>16</v>
       </c>
-      <c r="G6" s="38"/>
-      <c r="H6" s="39" t="s">
+      <c r="G6" s="42"/>
+      <c r="H6" s="37" t="s">
         <v>17</v>
       </c>
-      <c r="I6" s="39"/>
-      <c r="J6" s="40"/>
-      <c r="K6" s="40"/>
-      <c r="L6" s="40"/>
-      <c r="M6" s="40"/>
+      <c r="I6" s="37"/>
+      <c r="J6" s="43"/>
+      <c r="K6" s="43"/>
+      <c r="L6" s="43"/>
+      <c r="M6" s="43"/>
     </row>
     <row r="7" spans="1:26" ht="207.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="4">
@@ -2696,18 +2681,18 @@
       <c r="E7" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F7" s="38" t="s">
+      <c r="F7" s="42" t="s">
         <v>22</v>
       </c>
-      <c r="G7" s="38"/>
-      <c r="H7" s="39" t="s">
+      <c r="G7" s="42"/>
+      <c r="H7" s="37" t="s">
         <v>17</v>
       </c>
-      <c r="I7" s="39"/>
-      <c r="J7" s="40"/>
-      <c r="K7" s="40"/>
-      <c r="L7" s="40"/>
-      <c r="M7" s="40"/>
+      <c r="I7" s="37"/>
+      <c r="J7" s="43"/>
+      <c r="K7" s="43"/>
+      <c r="L7" s="43"/>
+      <c r="M7" s="43"/>
     </row>
     <row r="8" spans="1:26" ht="208.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="4">
@@ -2725,18 +2710,18 @@
       <c r="E8" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F8" s="39" t="s">
+      <c r="F8" s="37" t="s">
         <v>26</v>
       </c>
-      <c r="G8" s="39"/>
-      <c r="H8" s="39" t="s">
+      <c r="G8" s="37"/>
+      <c r="H8" s="37" t="s">
         <v>17</v>
       </c>
-      <c r="I8" s="39"/>
-      <c r="J8" s="40"/>
-      <c r="K8" s="40"/>
-      <c r="L8" s="40"/>
-      <c r="M8" s="40"/>
+      <c r="I8" s="37"/>
+      <c r="J8" s="43"/>
+      <c r="K8" s="43"/>
+      <c r="L8" s="43"/>
+      <c r="M8" s="43"/>
     </row>
     <row r="9" spans="1:26" ht="208.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="4">
@@ -2754,18 +2739,18 @@
       <c r="E9" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F9" s="38" t="s">
+      <c r="F9" s="42" t="s">
         <v>30</v>
       </c>
-      <c r="G9" s="38"/>
-      <c r="H9" s="39" t="s">
+      <c r="G9" s="42"/>
+      <c r="H9" s="37" t="s">
         <v>17</v>
       </c>
-      <c r="I9" s="39"/>
-      <c r="J9" s="41"/>
-      <c r="K9" s="41"/>
-      <c r="L9" s="41"/>
-      <c r="M9" s="41"/>
+      <c r="I9" s="37"/>
+      <c r="J9" s="38"/>
+      <c r="K9" s="38"/>
+      <c r="L9" s="38"/>
+      <c r="M9" s="38"/>
     </row>
     <row r="10" spans="1:26" ht="208.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="4">
@@ -2783,18 +2768,18 @@
       <c r="E10" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F10" s="38" t="s">
+      <c r="F10" s="42" t="s">
         <v>30</v>
       </c>
-      <c r="G10" s="38"/>
-      <c r="H10" s="39" t="s">
+      <c r="G10" s="42"/>
+      <c r="H10" s="37" t="s">
         <v>17</v>
       </c>
-      <c r="I10" s="39"/>
-      <c r="J10" s="41"/>
-      <c r="K10" s="41"/>
-      <c r="L10" s="41"/>
-      <c r="M10" s="41"/>
+      <c r="I10" s="37"/>
+      <c r="J10" s="38"/>
+      <c r="K10" s="38"/>
+      <c r="L10" s="38"/>
+      <c r="M10" s="38"/>
     </row>
     <row r="11" spans="1:26" ht="208.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="4">
@@ -2812,18 +2797,18 @@
       <c r="E11" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F11" s="39" t="s">
+      <c r="F11" s="37" t="s">
         <v>36</v>
       </c>
-      <c r="G11" s="39"/>
-      <c r="H11" s="39" t="s">
+      <c r="G11" s="37"/>
+      <c r="H11" s="37" t="s">
         <v>17</v>
       </c>
-      <c r="I11" s="39"/>
-      <c r="J11" s="41"/>
-      <c r="K11" s="41"/>
-      <c r="L11" s="41"/>
-      <c r="M11" s="41"/>
+      <c r="I11" s="37"/>
+      <c r="J11" s="38"/>
+      <c r="K11" s="38"/>
+      <c r="L11" s="38"/>
+      <c r="M11" s="38"/>
     </row>
     <row r="12" spans="1:26" ht="208.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="4">
@@ -2841,54 +2826,54 @@
       <c r="E12" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F12" s="39" t="s">
+      <c r="F12" s="37" t="s">
         <v>36</v>
       </c>
-      <c r="G12" s="39"/>
-      <c r="H12" s="39" t="s">
+      <c r="G12" s="37"/>
+      <c r="H12" s="37" t="s">
         <v>17</v>
       </c>
-      <c r="I12" s="39"/>
-      <c r="J12" s="41"/>
-      <c r="K12" s="41"/>
-      <c r="L12" s="41"/>
-      <c r="M12" s="41"/>
+      <c r="I12" s="37"/>
+      <c r="J12" s="38"/>
+      <c r="K12" s="38"/>
+      <c r="L12" s="38"/>
+      <c r="M12" s="38"/>
     </row>
     <row r="13" spans="1:26" ht="69" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A13" s="43" t="s">
+      <c r="A13" s="39" t="s">
         <v>39</v>
       </c>
-      <c r="B13" s="43"/>
-      <c r="C13" s="43"/>
-      <c r="D13" s="43"/>
-      <c r="E13" s="43"/>
-      <c r="F13" s="43"/>
-      <c r="G13" s="43"/>
-      <c r="H13" s="43"/>
-      <c r="I13" s="43"/>
-      <c r="J13" s="43"/>
-      <c r="K13" s="43"/>
-      <c r="L13" s="43"/>
-      <c r="M13" s="43"/>
+      <c r="B13" s="39"/>
+      <c r="C13" s="39"/>
+      <c r="D13" s="39"/>
+      <c r="E13" s="39"/>
+      <c r="F13" s="39"/>
+      <c r="G13" s="39"/>
+      <c r="H13" s="39"/>
+      <c r="I13" s="39"/>
+      <c r="J13" s="39"/>
+      <c r="K13" s="39"/>
+      <c r="L13" s="39"/>
+      <c r="M13" s="39"/>
     </row>
     <row r="14" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A14" s="44" t="s">
+      <c r="A14" s="40" t="s">
         <v>40</v>
       </c>
-      <c r="B14" s="44"/>
-      <c r="C14" s="44"/>
-      <c r="D14" s="44"/>
-      <c r="E14" s="44"/>
-      <c r="F14" s="45" t="s">
+      <c r="B14" s="40"/>
+      <c r="C14" s="40"/>
+      <c r="D14" s="40"/>
+      <c r="E14" s="40"/>
+      <c r="F14" s="41" t="s">
         <v>41</v>
       </c>
-      <c r="G14" s="45"/>
-      <c r="H14" s="45"/>
-      <c r="I14" s="45"/>
-      <c r="J14" s="45"/>
-      <c r="K14" s="45"/>
-      <c r="L14" s="45"/>
-      <c r="M14" s="45"/>
+      <c r="G14" s="41"/>
+      <c r="H14" s="41"/>
+      <c r="I14" s="41"/>
+      <c r="J14" s="41"/>
+      <c r="K14" s="41"/>
+      <c r="L14" s="41"/>
+      <c r="M14" s="41"/>
       <c r="N14" s="12"/>
       <c r="O14" s="12"/>
       <c r="P14" s="12"/>
@@ -2904,23 +2889,23 @@
       <c r="Z14" s="12"/>
     </row>
     <row r="15" spans="1:26" ht="81" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A15" s="42" t="s">
+      <c r="A15" s="36" t="s">
         <v>42</v>
       </c>
-      <c r="B15" s="42"/>
-      <c r="C15" s="42"/>
-      <c r="D15" s="42"/>
-      <c r="E15" s="42"/>
-      <c r="F15" s="42" t="s">
+      <c r="B15" s="36"/>
+      <c r="C15" s="36"/>
+      <c r="D15" s="36"/>
+      <c r="E15" s="36"/>
+      <c r="F15" s="36" t="s">
         <v>43</v>
       </c>
-      <c r="G15" s="42"/>
-      <c r="H15" s="42"/>
-      <c r="I15" s="42"/>
-      <c r="J15" s="42"/>
-      <c r="K15" s="42"/>
-      <c r="L15" s="42"/>
-      <c r="M15" s="42"/>
+      <c r="G15" s="36"/>
+      <c r="H15" s="36"/>
+      <c r="I15" s="36"/>
+      <c r="J15" s="36"/>
+      <c r="K15" s="36"/>
+      <c r="L15" s="36"/>
+      <c r="M15" s="36"/>
     </row>
     <row r="16" spans="1:26" ht="30.75" customHeight="1" x14ac:dyDescent="0.15"/>
     <row r="17" ht="52.5" customHeight="1" x14ac:dyDescent="0.15"/>
@@ -3900,6 +3885,35 @@
     <row r="991" ht="13.5" customHeight="1" x14ac:dyDescent="0.15"/>
   </sheetData>
   <mergeCells count="37">
+    <mergeCell ref="A1:M1"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="F2:M2"/>
+    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="F3:M3"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="H4:I4"/>
+    <mergeCell ref="J4:M4"/>
+    <mergeCell ref="F5:G5"/>
+    <mergeCell ref="H5:I5"/>
+    <mergeCell ref="J5:M5"/>
+    <mergeCell ref="F6:G6"/>
+    <mergeCell ref="H6:I6"/>
+    <mergeCell ref="J6:M6"/>
+    <mergeCell ref="F7:G7"/>
+    <mergeCell ref="H7:I7"/>
+    <mergeCell ref="J7:M7"/>
+    <mergeCell ref="F8:G8"/>
+    <mergeCell ref="H8:I8"/>
+    <mergeCell ref="J8:M8"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="H9:I9"/>
+    <mergeCell ref="J9:M9"/>
+    <mergeCell ref="F10:G10"/>
+    <mergeCell ref="H10:I10"/>
+    <mergeCell ref="J10:M10"/>
+    <mergeCell ref="F11:G11"/>
+    <mergeCell ref="H11:I11"/>
+    <mergeCell ref="J11:M11"/>
     <mergeCell ref="A15:E15"/>
     <mergeCell ref="F15:M15"/>
     <mergeCell ref="F12:G12"/>
@@ -3908,35 +3922,6 @@
     <mergeCell ref="A13:M13"/>
     <mergeCell ref="A14:E14"/>
     <mergeCell ref="F14:M14"/>
-    <mergeCell ref="F10:G10"/>
-    <mergeCell ref="H10:I10"/>
-    <mergeCell ref="J10:M10"/>
-    <mergeCell ref="F11:G11"/>
-    <mergeCell ref="H11:I11"/>
-    <mergeCell ref="J11:M11"/>
-    <mergeCell ref="F8:G8"/>
-    <mergeCell ref="H8:I8"/>
-    <mergeCell ref="J8:M8"/>
-    <mergeCell ref="F9:G9"/>
-    <mergeCell ref="H9:I9"/>
-    <mergeCell ref="J9:M9"/>
-    <mergeCell ref="F6:G6"/>
-    <mergeCell ref="H6:I6"/>
-    <mergeCell ref="J6:M6"/>
-    <mergeCell ref="F7:G7"/>
-    <mergeCell ref="H7:I7"/>
-    <mergeCell ref="J7:M7"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="H4:I4"/>
-    <mergeCell ref="J4:M4"/>
-    <mergeCell ref="F5:G5"/>
-    <mergeCell ref="H5:I5"/>
-    <mergeCell ref="J5:M5"/>
-    <mergeCell ref="A1:M1"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="F2:M2"/>
-    <mergeCell ref="A3:E3"/>
-    <mergeCell ref="F3:M3"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.23611111111111099" right="0.23611111111111099" top="0.74791666666666701" bottom="0.74791666666666701" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Agregando exportacion de bitacoras de mantenimiento
</commit_message>
<xml_diff>
--- a/public/plantillas/11_PROG_UTILIZACION.xlsx
+++ b/public/plantillas/11_PROG_UTILIZACION.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ventura/Desktop/Programacion/recal-hse/public/plantillas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A43E844-1FB9-3C42-BD7D-EB305A9EF62F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30025930-D121-0F4B-A695-6300E3A09CAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="33600" windowHeight="21000" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,7 +17,6 @@
     <sheet name="MANTENIMIENTO MARZO 2024" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'MANTENIMIENTO FEBRERO 2024'!$A$1:$H$8</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'MANTENIMIENTO MARZO 2024'!$A$1:$M$16</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'MANTENIMIENTO FEBRERO 2024'!$1:$4</definedName>
   </definedNames>
@@ -42,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="55">
   <si>
     <t>PROGRAMA DE UTILIZACIÓN DE MAQUINARIA Y EQUIPO</t>
   </si>
@@ -186,16 +185,6 @@
     <t>NUMERO ECONOMICO</t>
   </si>
   <si>
-    <t>ELABORO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-OBSERVACIONES:</t>
-  </si>
-  <si>
-    <t>OSVALDO JIMENEZ MORALES</t>
-  </si>
-  <si>
     <t xml:space="preserve">FECHA: </t>
   </si>
   <si>
@@ -212,6 +201,12 @@
   </si>
   <si>
     <t>BAJA DE OBRA</t>
+  </si>
+  <si>
+    <t>ELABORÓ</t>
+  </si>
+  <si>
+    <t>OBSERVACIONES:</t>
   </si>
 </sst>
 </file>
@@ -375,7 +370,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="11">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -503,11 +498,31 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -570,21 +585,40 @@
     <xf numFmtId="0" fontId="13" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -612,15 +646,36 @@
     <xf numFmtId="0" fontId="16" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -630,26 +685,8 @@
     <xf numFmtId="0" fontId="8" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1383,42 +1420,42 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:21" ht="60" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A1" s="27" t="s">
-        <v>52</v>
-      </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
-      <c r="E1" s="27"/>
-      <c r="F1" s="27"/>
-      <c r="G1" s="27"/>
-      <c r="H1" s="27"/>
+      <c r="A1" s="34" t="s">
+        <v>49</v>
+      </c>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="34"/>
+      <c r="F1" s="34"/>
+      <c r="G1" s="34"/>
+      <c r="H1" s="34"/>
     </row>
     <row r="2" spans="1:21" ht="27" x14ac:dyDescent="0.15">
-      <c r="A2" s="33" t="s">
-        <v>53</v>
-      </c>
-      <c r="B2" s="34"/>
-      <c r="C2" s="34"/>
-      <c r="D2" s="35"/>
-      <c r="E2" s="28" t="s">
+      <c r="A2" s="40" t="s">
         <v>50</v>
       </c>
-      <c r="F2" s="29"/>
-      <c r="G2" s="29"/>
-      <c r="H2" s="29"/>
+      <c r="B2" s="41"/>
+      <c r="C2" s="41"/>
+      <c r="D2" s="42"/>
+      <c r="E2" s="35" t="s">
+        <v>47</v>
+      </c>
+      <c r="F2" s="36"/>
+      <c r="G2" s="36"/>
+      <c r="H2" s="36"/>
     </row>
     <row r="3" spans="1:21" ht="49" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A3" s="28" t="s">
+      <c r="A3" s="35" t="s">
         <v>45</v>
       </c>
-      <c r="B3" s="29"/>
-      <c r="C3" s="29"/>
-      <c r="D3" s="32"/>
-      <c r="E3" s="30"/>
-      <c r="F3" s="31"/>
-      <c r="G3" s="31"/>
-      <c r="H3" s="31"/>
+      <c r="B3" s="36"/>
+      <c r="C3" s="36"/>
+      <c r="D3" s="39"/>
+      <c r="E3" s="37"/>
+      <c r="F3" s="38"/>
+      <c r="G3" s="38"/>
+      <c r="H3" s="38"/>
     </row>
     <row r="4" spans="1:21" ht="50" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="13" t="s">
@@ -1437,13 +1474,13 @@
         <v>46</v>
       </c>
       <c r="F4" s="15" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="G4" s="15" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="H4" s="18" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
     </row>
     <row r="5" spans="1:21" ht="157" customHeight="1" x14ac:dyDescent="0.15">
@@ -1457,28 +1494,30 @@
       <c r="H5" s="16"/>
     </row>
     <row r="6" spans="1:21" ht="69" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A6" s="22" t="s">
-        <v>48</v>
-      </c>
-      <c r="B6" s="22"/>
-      <c r="C6" s="22"/>
-      <c r="D6" s="22"/>
-      <c r="E6" s="22"/>
-      <c r="F6" s="22"/>
-      <c r="G6" s="22"/>
-      <c r="H6" s="22"/>
+      <c r="A6" s="56" t="s">
+        <v>54</v>
+      </c>
+      <c r="B6" s="23"/>
+      <c r="C6" s="23"/>
+      <c r="D6" s="23"/>
+      <c r="E6" s="23"/>
+      <c r="F6" s="23"/>
+      <c r="G6" s="23"/>
+      <c r="H6" s="24"/>
     </row>
     <row r="7" spans="1:21" ht="13.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A7" s="23" t="s">
-        <v>47</v>
-      </c>
-      <c r="B7" s="24"/>
-      <c r="C7" s="24"/>
-      <c r="D7" s="24"/>
-      <c r="E7" s="24"/>
-      <c r="F7" s="24"/>
-      <c r="G7" s="24"/>
-      <c r="H7" s="24"/>
+      <c r="A7" s="25"/>
+      <c r="B7" s="26"/>
+      <c r="C7" s="27" t="s">
+        <v>53</v>
+      </c>
+      <c r="D7" s="26"/>
+      <c r="E7" s="25"/>
+      <c r="F7" s="28" t="s">
+        <v>41</v>
+      </c>
+      <c r="G7" s="26"/>
+      <c r="H7" s="33"/>
       <c r="J7" s="12"/>
       <c r="K7" s="12"/>
       <c r="L7" s="12"/>
@@ -1493,16 +1532,14 @@
       <c r="U7" s="12"/>
     </row>
     <row r="8" spans="1:21" ht="81" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="25" t="s">
-        <v>49</v>
-      </c>
-      <c r="B8" s="26"/>
-      <c r="C8" s="26"/>
-      <c r="D8" s="26"/>
-      <c r="E8" s="26"/>
-      <c r="F8" s="26"/>
-      <c r="G8" s="26"/>
-      <c r="H8" s="26"/>
+      <c r="A8" s="29"/>
+      <c r="B8" s="30"/>
+      <c r="C8" s="22"/>
+      <c r="D8" s="31"/>
+      <c r="E8" s="29"/>
+      <c r="F8" s="32"/>
+      <c r="G8" s="30"/>
+      <c r="H8" s="31"/>
     </row>
     <row r="9" spans="1:21" ht="30.75" customHeight="1" x14ac:dyDescent="0.15"/>
     <row r="10" spans="1:21" ht="52.5" customHeight="1" x14ac:dyDescent="0.15"/>
@@ -2481,10 +2518,7 @@
     <row r="983" ht="13.5" customHeight="1" x14ac:dyDescent="0.15"/>
     <row r="984" ht="13.5" customHeight="1" x14ac:dyDescent="0.15"/>
   </sheetData>
-  <mergeCells count="8">
-    <mergeCell ref="A6:H6"/>
-    <mergeCell ref="A7:H7"/>
-    <mergeCell ref="A8:H8"/>
+  <mergeCells count="5">
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="E2:H2"/>
     <mergeCell ref="E3:H3"/>
@@ -2522,59 +2556,59 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="60" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="34" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
-      <c r="E1" s="27"/>
-      <c r="F1" s="27"/>
-      <c r="G1" s="27"/>
-      <c r="H1" s="27"/>
-      <c r="I1" s="27"/>
-      <c r="J1" s="27"/>
-      <c r="K1" s="27"/>
-      <c r="L1" s="27"/>
-      <c r="M1" s="27"/>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="34"/>
+      <c r="F1" s="34"/>
+      <c r="G1" s="34"/>
+      <c r="H1" s="34"/>
+      <c r="I1" s="34"/>
+      <c r="J1" s="34"/>
+      <c r="K1" s="34"/>
+      <c r="L1" s="34"/>
+      <c r="M1" s="34"/>
     </row>
     <row r="2" spans="1:26" ht="20" x14ac:dyDescent="0.15">
-      <c r="A2" s="46" t="s">
+      <c r="A2" s="43" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="46"/>
-      <c r="C2" s="46"/>
-      <c r="D2" s="46"/>
-      <c r="E2" s="46"/>
-      <c r="F2" s="47" t="s">
+      <c r="B2" s="43"/>
+      <c r="C2" s="43"/>
+      <c r="D2" s="43"/>
+      <c r="E2" s="43"/>
+      <c r="F2" s="44" t="s">
         <v>44</v>
       </c>
-      <c r="G2" s="47"/>
-      <c r="H2" s="47"/>
-      <c r="I2" s="47"/>
-      <c r="J2" s="47"/>
-      <c r="K2" s="47"/>
-      <c r="L2" s="47"/>
-      <c r="M2" s="47"/>
+      <c r="G2" s="44"/>
+      <c r="H2" s="44"/>
+      <c r="I2" s="44"/>
+      <c r="J2" s="44"/>
+      <c r="K2" s="44"/>
+      <c r="L2" s="44"/>
+      <c r="M2" s="44"/>
     </row>
     <row r="3" spans="1:26" ht="26.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A3" s="46" t="s">
+      <c r="A3" s="43" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="46"/>
-      <c r="C3" s="46"/>
-      <c r="D3" s="46"/>
-      <c r="E3" s="46"/>
-      <c r="F3" s="48" t="s">
+      <c r="B3" s="43"/>
+      <c r="C3" s="43"/>
+      <c r="D3" s="43"/>
+      <c r="E3" s="43"/>
+      <c r="F3" s="45" t="s">
         <v>3</v>
       </c>
-      <c r="G3" s="48"/>
-      <c r="H3" s="48"/>
-      <c r="I3" s="48"/>
-      <c r="J3" s="48"/>
-      <c r="K3" s="48"/>
-      <c r="L3" s="48"/>
-      <c r="M3" s="48"/>
+      <c r="G3" s="45"/>
+      <c r="H3" s="45"/>
+      <c r="I3" s="45"/>
+      <c r="J3" s="45"/>
+      <c r="K3" s="45"/>
+      <c r="L3" s="45"/>
+      <c r="M3" s="45"/>
     </row>
     <row r="4" spans="1:26" ht="36.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="2" t="s">
@@ -2592,20 +2626,20 @@
       <c r="E4" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="F4" s="44" t="s">
+      <c r="F4" s="46" t="s">
         <v>9</v>
       </c>
-      <c r="G4" s="44"/>
-      <c r="H4" s="44" t="s">
+      <c r="G4" s="46"/>
+      <c r="H4" s="46" t="s">
         <v>10</v>
       </c>
-      <c r="I4" s="44"/>
-      <c r="J4" s="45" t="s">
+      <c r="I4" s="46"/>
+      <c r="J4" s="47" t="s">
         <v>11</v>
       </c>
-      <c r="K4" s="45"/>
-      <c r="L4" s="45"/>
-      <c r="M4" s="45"/>
+      <c r="K4" s="47"/>
+      <c r="L4" s="47"/>
+      <c r="M4" s="47"/>
     </row>
     <row r="5" spans="1:26" ht="207.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="4">
@@ -2623,18 +2657,18 @@
       <c r="E5" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F5" s="42" t="s">
+      <c r="F5" s="48" t="s">
         <v>16</v>
       </c>
-      <c r="G5" s="42"/>
-      <c r="H5" s="37" t="s">
+      <c r="G5" s="48"/>
+      <c r="H5" s="49" t="s">
         <v>17</v>
       </c>
-      <c r="I5" s="37"/>
-      <c r="J5" s="43"/>
-      <c r="K5" s="43"/>
-      <c r="L5" s="43"/>
-      <c r="M5" s="43"/>
+      <c r="I5" s="49"/>
+      <c r="J5" s="50"/>
+      <c r="K5" s="50"/>
+      <c r="L5" s="50"/>
+      <c r="M5" s="50"/>
     </row>
     <row r="6" spans="1:26" ht="207.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="4">
@@ -2652,18 +2686,18 @@
       <c r="E6" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F6" s="42" t="s">
+      <c r="F6" s="48" t="s">
         <v>16</v>
       </c>
-      <c r="G6" s="42"/>
-      <c r="H6" s="37" t="s">
+      <c r="G6" s="48"/>
+      <c r="H6" s="49" t="s">
         <v>17</v>
       </c>
-      <c r="I6" s="37"/>
-      <c r="J6" s="43"/>
-      <c r="K6" s="43"/>
-      <c r="L6" s="43"/>
-      <c r="M6" s="43"/>
+      <c r="I6" s="49"/>
+      <c r="J6" s="50"/>
+      <c r="K6" s="50"/>
+      <c r="L6" s="50"/>
+      <c r="M6" s="50"/>
     </row>
     <row r="7" spans="1:26" ht="207.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="4">
@@ -2681,18 +2715,18 @@
       <c r="E7" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F7" s="42" t="s">
+      <c r="F7" s="48" t="s">
         <v>22</v>
       </c>
-      <c r="G7" s="42"/>
-      <c r="H7" s="37" t="s">
+      <c r="G7" s="48"/>
+      <c r="H7" s="49" t="s">
         <v>17</v>
       </c>
-      <c r="I7" s="37"/>
-      <c r="J7" s="43"/>
-      <c r="K7" s="43"/>
-      <c r="L7" s="43"/>
-      <c r="M7" s="43"/>
+      <c r="I7" s="49"/>
+      <c r="J7" s="50"/>
+      <c r="K7" s="50"/>
+      <c r="L7" s="50"/>
+      <c r="M7" s="50"/>
     </row>
     <row r="8" spans="1:26" ht="208.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="4">
@@ -2710,18 +2744,18 @@
       <c r="E8" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F8" s="37" t="s">
+      <c r="F8" s="49" t="s">
         <v>26</v>
       </c>
-      <c r="G8" s="37"/>
-      <c r="H8" s="37" t="s">
+      <c r="G8" s="49"/>
+      <c r="H8" s="49" t="s">
         <v>17</v>
       </c>
-      <c r="I8" s="37"/>
-      <c r="J8" s="43"/>
-      <c r="K8" s="43"/>
-      <c r="L8" s="43"/>
-      <c r="M8" s="43"/>
+      <c r="I8" s="49"/>
+      <c r="J8" s="50"/>
+      <c r="K8" s="50"/>
+      <c r="L8" s="50"/>
+      <c r="M8" s="50"/>
     </row>
     <row r="9" spans="1:26" ht="208.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="4">
@@ -2739,18 +2773,18 @@
       <c r="E9" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F9" s="42" t="s">
+      <c r="F9" s="48" t="s">
         <v>30</v>
       </c>
-      <c r="G9" s="42"/>
-      <c r="H9" s="37" t="s">
+      <c r="G9" s="48"/>
+      <c r="H9" s="49" t="s">
         <v>17</v>
       </c>
-      <c r="I9" s="37"/>
-      <c r="J9" s="38"/>
-      <c r="K9" s="38"/>
-      <c r="L9" s="38"/>
-      <c r="M9" s="38"/>
+      <c r="I9" s="49"/>
+      <c r="J9" s="51"/>
+      <c r="K9" s="51"/>
+      <c r="L9" s="51"/>
+      <c r="M9" s="51"/>
     </row>
     <row r="10" spans="1:26" ht="208.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="4">
@@ -2768,18 +2802,18 @@
       <c r="E10" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F10" s="42" t="s">
+      <c r="F10" s="48" t="s">
         <v>30</v>
       </c>
-      <c r="G10" s="42"/>
-      <c r="H10" s="37" t="s">
+      <c r="G10" s="48"/>
+      <c r="H10" s="49" t="s">
         <v>17</v>
       </c>
-      <c r="I10" s="37"/>
-      <c r="J10" s="38"/>
-      <c r="K10" s="38"/>
-      <c r="L10" s="38"/>
-      <c r="M10" s="38"/>
+      <c r="I10" s="49"/>
+      <c r="J10" s="51"/>
+      <c r="K10" s="51"/>
+      <c r="L10" s="51"/>
+      <c r="M10" s="51"/>
     </row>
     <row r="11" spans="1:26" ht="208.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="4">
@@ -2797,18 +2831,18 @@
       <c r="E11" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F11" s="37" t="s">
+      <c r="F11" s="49" t="s">
         <v>36</v>
       </c>
-      <c r="G11" s="37"/>
-      <c r="H11" s="37" t="s">
+      <c r="G11" s="49"/>
+      <c r="H11" s="49" t="s">
         <v>17</v>
       </c>
-      <c r="I11" s="37"/>
-      <c r="J11" s="38"/>
-      <c r="K11" s="38"/>
-      <c r="L11" s="38"/>
-      <c r="M11" s="38"/>
+      <c r="I11" s="49"/>
+      <c r="J11" s="51"/>
+      <c r="K11" s="51"/>
+      <c r="L11" s="51"/>
+      <c r="M11" s="51"/>
     </row>
     <row r="12" spans="1:26" ht="208.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="4">
@@ -2826,54 +2860,54 @@
       <c r="E12" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F12" s="37" t="s">
+      <c r="F12" s="49" t="s">
         <v>36</v>
       </c>
-      <c r="G12" s="37"/>
-      <c r="H12" s="37" t="s">
+      <c r="G12" s="49"/>
+      <c r="H12" s="49" t="s">
         <v>17</v>
       </c>
-      <c r="I12" s="37"/>
-      <c r="J12" s="38"/>
-      <c r="K12" s="38"/>
-      <c r="L12" s="38"/>
-      <c r="M12" s="38"/>
+      <c r="I12" s="49"/>
+      <c r="J12" s="51"/>
+      <c r="K12" s="51"/>
+      <c r="L12" s="51"/>
+      <c r="M12" s="51"/>
     </row>
     <row r="13" spans="1:26" ht="69" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="53" t="s">
         <v>39</v>
       </c>
-      <c r="B13" s="39"/>
-      <c r="C13" s="39"/>
-      <c r="D13" s="39"/>
-      <c r="E13" s="39"/>
-      <c r="F13" s="39"/>
-      <c r="G13" s="39"/>
-      <c r="H13" s="39"/>
-      <c r="I13" s="39"/>
-      <c r="J13" s="39"/>
-      <c r="K13" s="39"/>
-      <c r="L13" s="39"/>
-      <c r="M13" s="39"/>
+      <c r="B13" s="53"/>
+      <c r="C13" s="53"/>
+      <c r="D13" s="53"/>
+      <c r="E13" s="53"/>
+      <c r="F13" s="53"/>
+      <c r="G13" s="53"/>
+      <c r="H13" s="53"/>
+      <c r="I13" s="53"/>
+      <c r="J13" s="53"/>
+      <c r="K13" s="53"/>
+      <c r="L13" s="53"/>
+      <c r="M13" s="53"/>
     </row>
     <row r="14" spans="1:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A14" s="40" t="s">
+      <c r="A14" s="54" t="s">
         <v>40</v>
       </c>
-      <c r="B14" s="40"/>
-      <c r="C14" s="40"/>
-      <c r="D14" s="40"/>
-      <c r="E14" s="40"/>
-      <c r="F14" s="41" t="s">
+      <c r="B14" s="54"/>
+      <c r="C14" s="54"/>
+      <c r="D14" s="54"/>
+      <c r="E14" s="54"/>
+      <c r="F14" s="55" t="s">
         <v>41</v>
       </c>
-      <c r="G14" s="41"/>
-      <c r="H14" s="41"/>
-      <c r="I14" s="41"/>
-      <c r="J14" s="41"/>
-      <c r="K14" s="41"/>
-      <c r="L14" s="41"/>
-      <c r="M14" s="41"/>
+      <c r="G14" s="55"/>
+      <c r="H14" s="55"/>
+      <c r="I14" s="55"/>
+      <c r="J14" s="55"/>
+      <c r="K14" s="55"/>
+      <c r="L14" s="55"/>
+      <c r="M14" s="55"/>
       <c r="N14" s="12"/>
       <c r="O14" s="12"/>
       <c r="P14" s="12"/>
@@ -2889,23 +2923,23 @@
       <c r="Z14" s="12"/>
     </row>
     <row r="15" spans="1:26" ht="81" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A15" s="36" t="s">
+      <c r="A15" s="52" t="s">
         <v>42</v>
       </c>
-      <c r="B15" s="36"/>
-      <c r="C15" s="36"/>
-      <c r="D15" s="36"/>
-      <c r="E15" s="36"/>
-      <c r="F15" s="36" t="s">
+      <c r="B15" s="52"/>
+      <c r="C15" s="52"/>
+      <c r="D15" s="52"/>
+      <c r="E15" s="52"/>
+      <c r="F15" s="52" t="s">
         <v>43</v>
       </c>
-      <c r="G15" s="36"/>
-      <c r="H15" s="36"/>
-      <c r="I15" s="36"/>
-      <c r="J15" s="36"/>
-      <c r="K15" s="36"/>
-      <c r="L15" s="36"/>
-      <c r="M15" s="36"/>
+      <c r="G15" s="52"/>
+      <c r="H15" s="52"/>
+      <c r="I15" s="52"/>
+      <c r="J15" s="52"/>
+      <c r="K15" s="52"/>
+      <c r="L15" s="52"/>
+      <c r="M15" s="52"/>
     </row>
     <row r="16" spans="1:26" ht="30.75" customHeight="1" x14ac:dyDescent="0.15"/>
     <row r="17" ht="52.5" customHeight="1" x14ac:dyDescent="0.15"/>
@@ -3885,35 +3919,6 @@
     <row r="991" ht="13.5" customHeight="1" x14ac:dyDescent="0.15"/>
   </sheetData>
   <mergeCells count="37">
-    <mergeCell ref="A1:M1"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="F2:M2"/>
-    <mergeCell ref="A3:E3"/>
-    <mergeCell ref="F3:M3"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="H4:I4"/>
-    <mergeCell ref="J4:M4"/>
-    <mergeCell ref="F5:G5"/>
-    <mergeCell ref="H5:I5"/>
-    <mergeCell ref="J5:M5"/>
-    <mergeCell ref="F6:G6"/>
-    <mergeCell ref="H6:I6"/>
-    <mergeCell ref="J6:M6"/>
-    <mergeCell ref="F7:G7"/>
-    <mergeCell ref="H7:I7"/>
-    <mergeCell ref="J7:M7"/>
-    <mergeCell ref="F8:G8"/>
-    <mergeCell ref="H8:I8"/>
-    <mergeCell ref="J8:M8"/>
-    <mergeCell ref="F9:G9"/>
-    <mergeCell ref="H9:I9"/>
-    <mergeCell ref="J9:M9"/>
-    <mergeCell ref="F10:G10"/>
-    <mergeCell ref="H10:I10"/>
-    <mergeCell ref="J10:M10"/>
-    <mergeCell ref="F11:G11"/>
-    <mergeCell ref="H11:I11"/>
-    <mergeCell ref="J11:M11"/>
     <mergeCell ref="A15:E15"/>
     <mergeCell ref="F15:M15"/>
     <mergeCell ref="F12:G12"/>
@@ -3922,6 +3927,35 @@
     <mergeCell ref="A13:M13"/>
     <mergeCell ref="A14:E14"/>
     <mergeCell ref="F14:M14"/>
+    <mergeCell ref="F10:G10"/>
+    <mergeCell ref="H10:I10"/>
+    <mergeCell ref="J10:M10"/>
+    <mergeCell ref="F11:G11"/>
+    <mergeCell ref="H11:I11"/>
+    <mergeCell ref="J11:M11"/>
+    <mergeCell ref="F8:G8"/>
+    <mergeCell ref="H8:I8"/>
+    <mergeCell ref="J8:M8"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="H9:I9"/>
+    <mergeCell ref="J9:M9"/>
+    <mergeCell ref="F6:G6"/>
+    <mergeCell ref="H6:I6"/>
+    <mergeCell ref="J6:M6"/>
+    <mergeCell ref="F7:G7"/>
+    <mergeCell ref="H7:I7"/>
+    <mergeCell ref="J7:M7"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="H4:I4"/>
+    <mergeCell ref="J4:M4"/>
+    <mergeCell ref="F5:G5"/>
+    <mergeCell ref="H5:I5"/>
+    <mergeCell ref="J5:M5"/>
+    <mergeCell ref="A1:M1"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="F2:M2"/>
+    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="F3:M3"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.23611111111111099" right="0.23611111111111099" top="0.74791666666666701" bottom="0.74791666666666701" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>